<commit_message>
docs: add wsl2_freesurfer_vcxsrv_setup agent skill
</commit_message>
<xml_diff>
--- a/processed_data/test002/test002_ieegloc.xlsx
+++ b/processed_data/test002/test002_ieegloc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\seeg\Project_colorieeg_2026\processed_data\test002\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{828CD5D6-2F91-4D2C-95C6-540F6B6A9921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63AB0C1B-A2E0-4FF3-B577-19F2658F7DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JinYujia" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1368" uniqueCount="368">
   <si>
     <t>Channel</t>
   </si>
@@ -1126,6 +1126,10 @@
   </si>
   <si>
     <t>V2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Color_with_sti</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -2087,7 +2091,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T77"/>
+  <dimension ref="A1:T81"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="13" max="13" width="18" customWidth="1"/>
@@ -6867,6 +6871,254 @@
         <v>28</v>
       </c>
     </row>
+    <row r="78" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F78" s="3">
+        <v>0.52</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H78" s="3">
+        <v>0.52</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J78" s="3">
+        <v>0.52</v>
+      </c>
+      <c r="K78" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="L78" s="3">
+        <v>0.52</v>
+      </c>
+      <c r="M78" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="N78" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="O78" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="P78" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q78" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R78" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="S78" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="T78" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F79" s="3">
+        <v>0.69</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H79" s="3">
+        <v>0.69</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J79" s="3">
+        <v>0.69</v>
+      </c>
+      <c r="K79" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="L79" s="3">
+        <v>0.69</v>
+      </c>
+      <c r="M79" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="N79" s="3">
+        <v>0.46</v>
+      </c>
+      <c r="O79" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="P79" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q79" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R79" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="S79" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="T79" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F80" s="3">
+        <v>0.83</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H80" s="3">
+        <v>0.52</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J80" s="3">
+        <v>0.83</v>
+      </c>
+      <c r="K80" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="L80" s="3">
+        <v>0.63</v>
+      </c>
+      <c r="M80" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="N80" s="3">
+        <v>0.49</v>
+      </c>
+      <c r="O80" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="P80" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q80" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R80" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="S80" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T80" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>74</v>
+      </c>
+      <c r="B81" t="s">
+        <v>75</v>
+      </c>
+      <c r="C81" t="s">
+        <v>76</v>
+      </c>
+      <c r="D81" t="s">
+        <v>77</v>
+      </c>
+      <c r="E81" t="s">
+        <v>24</v>
+      </c>
+      <c r="F81" s="1">
+        <v>0.49</v>
+      </c>
+      <c r="G81" t="s">
+        <v>78</v>
+      </c>
+      <c r="H81" s="1">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="I81" t="s">
+        <v>78</v>
+      </c>
+      <c r="J81" s="1">
+        <v>0.32</v>
+      </c>
+      <c r="K81" t="s">
+        <v>26</v>
+      </c>
+      <c r="L81" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="M81" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="N81" s="1">
+        <v>1</v>
+      </c>
+      <c r="O81" t="s">
+        <v>79</v>
+      </c>
+      <c r="P81" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q81" t="s">
+        <v>79</v>
+      </c>
+      <c r="R81" t="s">
+        <v>28</v>
+      </c>
+      <c r="S81" t="s">
+        <v>28</v>
+      </c>
+      <c r="T81" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>